<commit_message>
Add 10-digit phone restriction, GPS location fetcher, and delivery address/pincode fields
</commit_message>
<xml_diff>
--- a/data/inquiries.xlsx
+++ b/data/inquiries.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -482,9 +482,44 @@
         <v>Verifying Excel sheet auto creation</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>6/8/2026, 9:20:49 am</v>
+      </c>
+      <c r="B3" t="str">
+        <v>VED-449657</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Ved</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Enterprises</v>
+      </c>
+      <c r="E3" t="str">
+        <v>8995898787</v>
+      </c>
+      <c r="F3" t="str">
+        <v>vedenterprises566@gmail.com</v>
+      </c>
+      <c r="G3" t="str">
+        <v>uoiiou</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Punjab (Ludhiana / Amritsar)</v>
+      </c>
+      <c r="I3" t="str">
+        <v>YES</v>
+      </c>
+      <c r="J3" t="str">
+        <v>MX Lurex 50/85 Fine Count (50/85 Fine Count): 100Kg; Space Polyester Yarn (300D - 550D) (300 Denier to 550 Denier): 100Kg; Poly Enigma Yarn 550 Denier (550 Denier): 100Kg; Stretch Yarn (Polyester Vislon) (Variable Stretch Counts): 100Kg</v>
+      </c>
+      <c r="K3" t="str">
+        <v>hiugu</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>